<commit_message>
feat: readable categorical ARDs + realistic DM example analyses
Add a ydisctools method-template overlay (merged over the vendored siera
catalog, same-id entries override) whose categorical_summary uses the
modern cards by=/variables= denominator pattern: generated ARDs now carry
the real category variable name and levels (variable = AGEGR1,
variable_level = '<65') instead of the legacy dummy placeholder, with
identical statistics. The parameter template and the shipped example set
now mirror a realistic DM display (big N, Age continuous, Age group 1/2,
Sex, Race, Ethnicity); examples regenerated, tests and the ARS-chain
article updated to the new ARD shape. Bump to 0.0.235.

Closes #16

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/ars-examples/ARS_dm_ae.xlsx
+++ b/inst/ars-examples/ARS_dm_ae.xlsx
@@ -385,7 +385,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ydisctools 0.0.233 build_ars()</t>
+          <t>ydisctools 0.0.234 build_ars()</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>n and percentage of a categorical analysis variable per group, with a referenced denominator analysis and a data-driven/pre-defined grouping branch. Verified against Common_Safety_Displays Mth01_CatVar_Summ_ByGrp; current cards API. Spurious by_vars/strata_vars params from the legacy sheet have been dropped (the template uses by_listc).</t>
+          <t>Distinct-subject n and percentage per category and group, with a referenced denominator analysis. Modern cards pattern: the category variable is passed as `variables=` (so it lands in the ARD's variable / variable_level columns) and the outer grouping(s) as `by=` (`strata=` when the innermost grouping is data-driven). ydisctools overlay entry; replaces the siera catalog's distinct+dummy template.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>n and percentage of a categorical analysis variable per group, with a referenced denominator analysis and a data-driven/pre-defined grouping branch. Verified against Common_Safety_Displays Mth01_CatVar_Summ_ByGrp; current cards API. Spurious by_vars/strata_vars params from the legacy sheet have been dropped (the template uses by_listc).</t>
+          <t>Distinct-subject n and percentage per category and group, with a referenced denominator analysis. Modern cards pattern: the category variable is passed as `variables=` (so it lands in the ARD's variable / variable_level columns) and the outer grouping(s) as `by=` (`strata=` when the innermost grouping is data-driven). ydisctools overlay entry; replaces the siera catalog's distinct+dummy template.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1070,25 +1070,22 @@
           <t>denom_dataset = df2_denomanaidhere |&gt;
   dplyr::select(denom_anagroupvarshere)
 in_data = df2_analysisidhere |&gt;
-    dplyr::distinct(distinctlisthere) |&gt;
-    dplyr::mutate(dummy = 'dummyvar')
+    dplyr::distinct(distinctlisthere)
 dataDriven = isdatadrivenhere
 if(dataDriven == TRUE){
 df3_analysisidhere &lt;-
   cards::ard_tabulate(
-    data = in_data,
-    strata = c(byvarshere),
-    variables = 'dummy',
+    data = in_data
+    stratavarshere,
     denominator = denom_dataset
   ) } else {
 df3_analysisidhere &lt;-
  cards::ard_tabulate(
-    data = in_data,
-    by = c(byvarshere),
-    variables = 'dummy',
+    data = in_data
+    byvarshere,
     denominator = denom_dataset
   ) }
-df3_analysisidhere &lt;- df3_analysisidhere|&gt;
+df3_analysisidhere &lt;- df3_analysisidhere |&gt;
   dplyr::filter(stat_name %in% c('n', 'p')) |&gt;
   dplyr::mutate(operationid = dplyr::case_when(stat_name == 'n' ~ 'opid1here',
                                                stat_name == 'p' ~ 'opid2here'))</t>
@@ -1102,7 +1099,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1393,17 +1390,44 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Grouping variables as a quoted, comma-separated list</t>
+          <t>by = outer grouping(s), variables = category variable</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>by vars (list)</t>
+          <t>by/variables args</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>by_listc</t>
+          <t>by_vars</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Mth_categorical_summary</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>stratavarshere</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>strata = outer grouping(s), variables = category variable</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>strata/variables args</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>strata_vars</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1472,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1588,7 +1612,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Age group, n (%)</t>
+          <t>Age group 1, n (%)</t>
         </is>
       </c>
       <c r="E5">
@@ -1616,7 +1640,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Sex, n (%)</t>
+          <t>Age group 2, n (%)</t>
         </is>
       </c>
       <c r="E6">
@@ -1644,7 +1668,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Race, n (%)</t>
+          <t>Sex, n (%)</t>
         </is>
       </c>
       <c r="E7">
@@ -1668,19 +1692,19 @@
         </is>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Summary of Treatment-Emergent Adverse Events</t>
+          <t>Race, n (%)</t>
         </is>
       </c>
       <c r="E8">
-        <v>2</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Out_ae</t>
+        <v>6</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>An_06</t>
         </is>
       </c>
     </row>
@@ -1700,15 +1724,15 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Number of subjects</t>
+          <t>Ethnicity, n (%)</t>
         </is>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>An_06</t>
+          <t>An_07</t>
         </is>
       </c>
     </row>
@@ -1724,19 +1748,19 @@
         </is>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Subjects with at least one TEAE, n (%)</t>
+          <t>Summary of Treatment-Emergent Adverse Events</t>
         </is>
       </c>
       <c r="E10">
         <v>2</v>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>An_07</t>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Out_ae</t>
         </is>
       </c>
     </row>
@@ -1756,11 +1780,11 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>TEAE by System Organ Class, n (%)</t>
+          <t>Number of subjects</t>
         </is>
       </c>
       <c r="E11">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1784,11 +1808,11 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>TEAE by Preferred Term, n (%)</t>
+          <t>Subjects with at least one TEAE, n (%)</t>
         </is>
       </c>
       <c r="E12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1812,15 +1836,71 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>TEAE by System Organ Class, n (%)</t>
+        </is>
+      </c>
+      <c r="E13">
+        <v>3</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>An_10</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>List of Planned Analyses</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>LOPA</t>
+        </is>
+      </c>
+      <c r="C14">
+        <v>2</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>TEAE by Preferred Term, n (%)</t>
+        </is>
+      </c>
+      <c r="E14">
+        <v>4</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>An_11</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>List of Planned Analyses</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LOPA</t>
+        </is>
+      </c>
+      <c r="C15">
+        <v>2</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>TEAE by severity, n (%)</t>
         </is>
       </c>
-      <c r="E13">
+      <c r="E15">
         <v>5</v>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>An_10</t>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>An_12</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2301,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2540,12 +2620,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AnlsGrp_03_SEX</t>
+          <t>AnlsGrp_03_AGEGR2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SEX</t>
+          <t>AGEGR2</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2555,7 +2635,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEX</t>
+          <t>AGEGR2</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2567,12 +2647,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AnlsGrp_04_RACE</t>
+          <t>AnlsGrp_04_SEX</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>RACE</t>
+          <t>SEX</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2582,7 +2662,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>RACE</t>
+          <t>SEX</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2594,22 +2674,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AnlsGrp_05_AEBODSYS</t>
+          <t>AnlsGrp_05_RACE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AEBODSYS</t>
+          <t>RACE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ADAE</t>
+          <t>ADSL</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AEBODSYS</t>
+          <t>RACE</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2621,22 +2701,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AnlsGrp_06_AEDECOD</t>
+          <t>AnlsGrp_06_ETHNIC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AEDECOD</t>
+          <t>ETHNIC</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ADAE</t>
+          <t>ADSL</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>AEDECOD</t>
+          <t>ETHNIC</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2648,25 +2728,79 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AnlsGrp_07_AESEV</t>
+          <t>AnlsGrp_07_AEBODSYS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>AEBODSYS</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ADAE</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>AEBODSYS</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AnlsGrp_08_AEDECOD</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>AEDECOD</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ADAE</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>AEDECOD</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AnlsGrp_09_AESEV</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>AESEV</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>ADAE</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>AESEV</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
@@ -2679,7 +2813,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:S13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2886,7 +3020,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Age group, n (%)</t>
+          <t>Age group 1, n (%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2962,7 +3096,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sex, n (%)</t>
+          <t>Age group 2, n (%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -2985,7 +3119,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>AnlsGrp_03_SEX</t>
+          <t>AnlsGrp_03_AGEGR2</t>
         </is>
       </c>
       <c r="K5" t="b">
@@ -3038,7 +3172,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Race, n (%)</t>
+          <t>Sex, n (%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -3061,7 +3195,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>AnlsGrp_04_RACE</t>
+          <t>AnlsGrp_04_SEX</t>
         </is>
       </c>
       <c r="K6" t="b">
@@ -3114,7 +3248,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Number of subjects</t>
+          <t>Race, n (%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -3135,6 +3269,14 @@
       <c r="I7" t="b">
         <v>1</v>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>AnlsGrp_05_RACE</t>
+        </is>
+      </c>
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
       <c r="M7" t="inlineStr">
         <is>
           <t>ADSL</t>
@@ -3147,7 +3289,27 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Mth_total_n</t>
+          <t>Mth_categorical_summary</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Mth_categorical_summary_pct_num</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>An_06</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Mth_categorical_summary_pct_den</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>An_01</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3324,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Subjects with at least one TEAE, n (%)</t>
+          <t>Ethnicity, n (%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -3183,14 +3345,17 @@
       <c r="I8" t="b">
         <v>1</v>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Dss_01</t>
-        </is>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>AnlsGrp_06_ETHNIC</t>
+        </is>
+      </c>
+      <c r="K8" t="b">
+        <v>1</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>ADAE</t>
+          <t>ADSL</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -3220,7 +3385,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>An_06</t>
+          <t>An_01</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3400,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>TEAE by System Organ Class, n (%)</t>
+          <t>Number of subjects</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -3256,22 +3421,9 @@
       <c r="I9" t="b">
         <v>1</v>
       </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>AnlsGrp_05_AEBODSYS</t>
-        </is>
-      </c>
-      <c r="K9" t="b">
-        <v>1</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Dss_01</t>
-        </is>
-      </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>ADAE</t>
+          <t>ADSL</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -3281,27 +3433,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Mth_categorical_summary</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Mth_categorical_summary_pct_num</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>An_08</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>Mth_categorical_summary_pct_den</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>An_06</t>
+          <t>Mth_total_n</t>
         </is>
       </c>
     </row>
@@ -3316,7 +3448,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>TEAE by Preferred Term, n (%)</t>
+          <t>Subjects with at least one TEAE, n (%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -3337,14 +3469,6 @@
       <c r="I10" t="b">
         <v>1</v>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>AnlsGrp_06_AEDECOD</t>
-        </is>
-      </c>
-      <c r="K10" t="b">
-        <v>1</v>
-      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>Dss_01</t>
@@ -3382,7 +3506,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>An_06</t>
+          <t>An_08</t>
         </is>
       </c>
     </row>
@@ -3397,73 +3521,235 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>TEAE by System Organ Class, n (%)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>SPECIFIED IN SAP</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>AnalysisSet_01</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>AnlsGrp_01_TRT01A</t>
+        </is>
+      </c>
+      <c r="I11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>AnlsGrp_07_AEBODSYS</t>
+        </is>
+      </c>
+      <c r="K11" t="b">
+        <v>1</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Dss_01</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>ADAE</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>USUBJID</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Mth_categorical_summary</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Mth_categorical_summary_pct_num</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>An_10</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Mth_categorical_summary_pct_den</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>An_08</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>An_11</t>
+        </is>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TEAE by Preferred Term, n (%)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SPECIFIED IN SAP</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>AnalysisSet_01</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>AnlsGrp_01_TRT01A</t>
+        </is>
+      </c>
+      <c r="I12" t="b">
+        <v>1</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>AnlsGrp_08_AEDECOD</t>
+        </is>
+      </c>
+      <c r="K12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Dss_01</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>ADAE</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>USUBJID</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Mth_categorical_summary</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Mth_categorical_summary_pct_num</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>An_11</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Mth_categorical_summary_pct_den</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>An_08</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>An_12</t>
+        </is>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>TEAE by severity, n (%)</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>SPECIFIED IN SAP</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>AnalysisSet_01</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>AnlsGrp_01_TRT01A</t>
         </is>
       </c>
-      <c r="I11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>AnlsGrp_07_AESEV</t>
-        </is>
-      </c>
-      <c r="K11" t="b">
-        <v>1</v>
-      </c>
-      <c r="L11" t="inlineStr">
+      <c r="I13" t="b">
+        <v>1</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>AnlsGrp_09_AESEV</t>
+        </is>
+      </c>
+      <c r="K13" t="b">
+        <v>1</v>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>Dss_01</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>ADAE</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>USUBJID</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>Mth_categorical_summary</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>Mth_categorical_summary_pct_num</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>An_10</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>An_12</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
         <is>
           <t>Mth_categorical_summary_pct_den</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>An_06</t>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>An_08</t>
         </is>
       </c>
     </row>

</xml_diff>